<commit_message>
Ajustes al Login y al Index (se quitaron unos script y se ajustó lallamad aal método logout
</commit_message>
<xml_diff>
--- a/DOC/Cronograma.xlsx
+++ b/DOC/Cronograma.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Desarrollo\IAM\DOC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D73EBA5-CC9A-4467-92DF-33F91EF9511A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F4B4396-7350-445C-B036-237CDBC512DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{53363212-2131-440C-80BA-64ED1C922C49}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
   <si>
     <t>Semana</t>
   </si>
@@ -44,13 +44,22 @@
   <si>
     <t>Fecha Fin</t>
   </si>
+  <si>
+    <t>Pase a producción</t>
+  </si>
+  <si>
+    <t>Vamos por acá</t>
+  </si>
+  <si>
+    <t>QA</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -87,16 +96,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -412,307 +427,376 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4295C26-BAF6-4CCA-83DC-1428FB768C84}">
-  <dimension ref="A1:C48"/>
+  <sheetPr codeName="Hoja1"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="1"/>
     <col min="2" max="2" width="27.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" s="4"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="2">
         <v>45775</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="5">
         <v>45781</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>45782</v>
+      </c>
+      <c r="C3" s="5">
+        <v>45788</v>
+      </c>
+      <c r="D3" s="5"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>45782</v>
-      </c>
-      <c r="C4" s="2">
-        <v>45788</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>45789</v>
+      </c>
+      <c r="C4" s="5">
+        <v>45795</v>
+      </c>
+      <c r="D4" s="5"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>45796</v>
+      </c>
+      <c r="C5" s="5">
+        <v>45802</v>
+      </c>
+      <c r="D5" s="5"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>45803</v>
+      </c>
+      <c r="C6" s="5">
+        <v>45809</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>45810</v>
+      </c>
+      <c r="C7" s="5">
+        <v>45816</v>
+      </c>
+      <c r="D7" s="5"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <v>45817</v>
+      </c>
+      <c r="C8" s="5">
+        <v>45823</v>
+      </c>
+      <c r="D8" s="5"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <v>45824</v>
+      </c>
+      <c r="C9" s="5">
+        <v>45830</v>
+      </c>
+      <c r="D9" s="5"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2">
+        <v>45831</v>
+      </c>
+      <c r="C10" s="5">
+        <v>45837</v>
+      </c>
+      <c r="D10" s="5"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2">
+        <v>45838</v>
+      </c>
+      <c r="C11" s="5">
+        <v>45844</v>
+      </c>
+      <c r="D11" s="5"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2">
+        <v>45845</v>
+      </c>
+      <c r="C12" s="5">
+        <v>45851</v>
+      </c>
+      <c r="D12" s="5"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <v>45852</v>
+      </c>
+      <c r="C13" s="5">
+        <v>45858</v>
+      </c>
+      <c r="D13" s="5"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2">
+        <v>45859</v>
+      </c>
+      <c r="C14" s="5">
+        <v>45865</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2">
+        <v>45866</v>
+      </c>
+      <c r="C15" s="5">
+        <v>45872</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2">
+        <v>45873</v>
+      </c>
+      <c r="C16" s="5">
+        <v>45879</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="2">
-        <v>45789</v>
-      </c>
-      <c r="C5" s="2">
-        <v>45795</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>4</v>
-      </c>
-      <c r="B6" s="2">
-        <v>45796</v>
-      </c>
-      <c r="C6" s="2">
-        <v>45802</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>5</v>
-      </c>
-      <c r="B7" s="2">
-        <v>45803</v>
-      </c>
-      <c r="C7" s="2">
-        <v>45809</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>6</v>
-      </c>
-      <c r="B8" s="2">
-        <v>45810</v>
-      </c>
-      <c r="C8" s="2">
-        <v>45816</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>7</v>
-      </c>
-      <c r="B9" s="2">
-        <v>45817</v>
-      </c>
-      <c r="C9" s="2">
-        <v>45823</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
-        <v>8</v>
-      </c>
-      <c r="B10" s="2">
-        <v>45824</v>
-      </c>
-      <c r="C10" s="2">
-        <v>45830</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
-        <v>9</v>
-      </c>
-      <c r="B11" s="2">
-        <v>45831</v>
-      </c>
-      <c r="C11" s="2">
-        <v>45837</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
-        <v>10</v>
-      </c>
-      <c r="B12" s="2">
-        <v>45838</v>
-      </c>
-      <c r="C12" s="2">
-        <v>45844</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
-        <v>11</v>
-      </c>
-      <c r="B13" s="2">
-        <v>45845</v>
-      </c>
-      <c r="C13" s="2">
-        <v>45851</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
-        <v>12</v>
-      </c>
-      <c r="B14" s="2">
-        <v>45852</v>
-      </c>
-      <c r="C14" s="2">
-        <v>45858</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
-        <v>13</v>
-      </c>
-      <c r="B15" s="2">
-        <v>45859</v>
-      </c>
-      <c r="C15" s="2">
-        <v>45865</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
-        <v>14</v>
-      </c>
-      <c r="B16" s="2">
-        <v>45866</v>
-      </c>
-      <c r="C16" s="2">
-        <v>45872</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
-        <v>15</v>
-      </c>
-      <c r="B17" s="2">
-        <v>45873</v>
-      </c>
-      <c r="C17" s="2">
-        <v>45879</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D20" s="2"/>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B22" s="2"/>
       <c r="C22" s="2"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="2"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D24" s="2"/>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D25" s="2"/>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D26" s="2"/>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D27" s="2"/>
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D28" s="2"/>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B29" s="2"/>
       <c r="C29" s="2"/>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D29" s="2"/>
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D30" s="2"/>
+    </row>
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D31" s="2"/>
+    </row>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
-    </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D32" s="2"/>
+    </row>
+    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
-    </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D33" s="2"/>
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-    </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D34" s="2"/>
+    </row>
+    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
-    </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D35" s="2"/>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
-    </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D36" s="2"/>
+    </row>
+    <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
-    </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D37" s="2"/>
+    </row>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B39" s="2"/>
-    </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+    </row>
+    <row r="40" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
-    </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D40" s="2"/>
+    </row>
+    <row r="41" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
-    </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D41" s="2"/>
+    </row>
+    <row r="42" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
-    </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
-    </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C44" s="2"/>
-    </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C45" s="2"/>
-    </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C47" s="2"/>
-    </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C48" s="2"/>
+      <c r="D42" s="2"/>
+    </row>
+    <row r="43" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D43" s="2"/>
+    </row>
+    <row r="44" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D44" s="2"/>
+    </row>
+    <row r="46" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D46" s="2"/>
+    </row>
+    <row r="47" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D47" s="2"/>
     </row>
   </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>